<commit_message>
Add deterministic 2-opt exchange and integrate VNS in main
Introduced a deterministic 2-opt exchange local search in busca_local.py and added print statements for better traceability. Updated main.py to integrate the VNS metaheuristic after local search phases, adjusting result handling and output. Minor comment and code improvements in metaheuristics.py for VNS neighborhood shaking.
</commit_message>
<xml_diff>
--- a/Resultados_atualizado.xlsx
+++ b/Resultados_atualizado.xlsx
@@ -508,16 +508,16 @@
         <v>236</v>
       </c>
       <c r="G2" t="n">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="H2" t="n">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2567415237426758</v>
+        <v>0.3388864994049072</v>
       </c>
       <c r="J2" t="n">
-        <v>2.11864406779661</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -554,7 +554,7 @@
         <v>238</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2627460956573486</v>
+        <v>0.2562170028686523</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>193</v>
       </c>
       <c r="G4" t="n">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="H4" t="n">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2425696849822998</v>
+        <v>0.2718319892883301</v>
       </c>
       <c r="J4" t="n">
-        <v>3.10880829015544</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -634,7 +634,7 @@
         <v>196</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2328448295593262</v>
+        <v>0.2291984558105469</v>
       </c>
       <c r="J5" t="n">
         <v>1.55440414507772</v>
@@ -668,16 +668,16 @@
         <v>336</v>
       </c>
       <c r="G6" t="n">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="H6" t="n">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2284045219421387</v>
+        <v>0.2349972724914551</v>
       </c>
       <c r="J6" t="n">
-        <v>1.488095238095238</v>
+        <v>0.2976190476190476</v>
       </c>
     </row>
     <row r="7">
@@ -708,16 +708,16 @@
         <v>338</v>
       </c>
       <c r="G7" t="n">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="H7" t="n">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2461073398590088</v>
+        <v>0.2507057189941406</v>
       </c>
       <c r="J7" t="n">
-        <v>1.775147928994083</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -754,7 +754,7 @@
         <v>296</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2775943279266357</v>
+        <v>0.2038760185241699</v>
       </c>
       <c r="J8" t="n">
         <v>1.718213058419244</v>
@@ -794,7 +794,7 @@
         <v>293</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2189638614654541</v>
+        <v>0.2400901317596436</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>361</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3946843147277832</v>
+        <v>0.4684712886810303</v>
       </c>
       <c r="J10" t="n">
         <v>1.690140845070422</v>
@@ -874,7 +874,7 @@
         <v>363</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3921210765838623</v>
+        <v>0.5461428165435791</v>
       </c>
       <c r="J11" t="n">
         <v>2.253521126760563</v>
@@ -914,7 +914,7 @@
         <v>293</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3785526752471924</v>
+        <v>0.5375795364379883</v>
       </c>
       <c r="J12" t="n">
         <v>2.807017543859649</v>
@@ -954,7 +954,7 @@
         <v>293</v>
       </c>
       <c r="I13" t="n">
-        <v>0.409123420715332</v>
+        <v>0.5643036365509033</v>
       </c>
       <c r="J13" t="n">
         <v>2.807017543859649</v>
@@ -988,16 +988,16 @@
         <v>505</v>
       </c>
       <c r="G14" t="n">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="H14" t="n">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="I14" t="n">
-        <v>0.4812803268432617</v>
+        <v>0.4822604656219482</v>
       </c>
       <c r="J14" t="n">
-        <v>1.386138613861386</v>
+        <v>1.782178217821782</v>
       </c>
     </row>
     <row r="15">
@@ -1028,16 +1028,16 @@
         <v>505</v>
       </c>
       <c r="G15" t="n">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="H15" t="n">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3811981678009033</v>
+        <v>0.6600596904754639</v>
       </c>
       <c r="J15" t="n">
-        <v>1.584158415841584</v>
+        <v>1.386138613861386</v>
       </c>
     </row>
     <row r="16">
@@ -1068,16 +1068,16 @@
         <v>435</v>
       </c>
       <c r="G16" t="n">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="H16" t="n">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="I16" t="n">
-        <v>0.3537452220916748</v>
+        <v>0.6848187446594238</v>
       </c>
       <c r="J16" t="n">
-        <v>1.379310344827586</v>
+        <v>0.9195402298850575</v>
       </c>
     </row>
     <row r="17">
@@ -1108,16 +1108,16 @@
         <v>435</v>
       </c>
       <c r="G17" t="n">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="H17" t="n">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="I17" t="n">
-        <v>0.4141130447387695</v>
+        <v>0.6449654102325439</v>
       </c>
       <c r="J17" t="n">
-        <v>1.839080459770115</v>
+        <v>1.379310344827586</v>
       </c>
     </row>
     <row r="18">
@@ -1148,16 +1148,16 @@
         <v>481</v>
       </c>
       <c r="G18" t="n">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="H18" t="n">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="I18" t="n">
-        <v>0.5649814605712891</v>
+        <v>0.9610354900360107</v>
       </c>
       <c r="J18" t="n">
-        <v>2.702702702702703</v>
+        <v>2.286902286902287</v>
       </c>
     </row>
     <row r="19">
@@ -1188,16 +1188,16 @@
         <v>481</v>
       </c>
       <c r="G19" t="n">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="H19" t="n">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="I19" t="n">
-        <v>0.5968625545501709</v>
+        <v>1.251049518585205</v>
       </c>
       <c r="J19" t="n">
-        <v>1.871101871101871</v>
+        <v>3.742203742203742</v>
       </c>
     </row>
     <row r="20">
@@ -1228,16 +1228,16 @@
         <v>386</v>
       </c>
       <c r="G20" t="n">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="H20" t="n">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6219789981842041</v>
+        <v>2.215589046478271</v>
       </c>
       <c r="J20" t="n">
-        <v>2.590673575129534</v>
+        <v>1.813471502590673</v>
       </c>
     </row>
     <row r="21">
@@ -1274,7 +1274,7 @@
         <v>399</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6433465480804443</v>
+        <v>1.601418972015381</v>
       </c>
       <c r="J21" t="n">
         <v>3.367875647668394</v>
@@ -1308,16 +1308,16 @@
         <v>681</v>
       </c>
       <c r="G22" t="n">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="H22" t="n">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="I22" t="n">
-        <v>0.5510501861572266</v>
+        <v>1.051834106445312</v>
       </c>
       <c r="J22" t="n">
-        <v>1.174743024963289</v>
+        <v>0.4405286343612335</v>
       </c>
     </row>
     <row r="23">
@@ -1348,16 +1348,16 @@
         <v>681</v>
       </c>
       <c r="G23" t="n">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="H23" t="n">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="I23" t="n">
-        <v>0.5554099082946777</v>
+        <v>2.00340461730957</v>
       </c>
       <c r="J23" t="n">
-        <v>1.174743024963289</v>
+        <v>0.881057268722467</v>
       </c>
     </row>
     <row r="24">
@@ -1394,7 +1394,7 @@
         <v>599</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5257449150085449</v>
+        <v>0.8289389610290527</v>
       </c>
       <c r="J24" t="n">
         <v>2.218430034129693</v>
@@ -1428,16 +1428,16 @@
         <v>586</v>
       </c>
       <c r="G25" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="H25" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="I25" t="n">
-        <v>0.6916337013244629</v>
+        <v>1.856411695480347</v>
       </c>
       <c r="J25" t="n">
-        <v>1.194539249146758</v>
+        <v>1.023890784982935</v>
       </c>
     </row>
     <row r="26">
@@ -1468,16 +1468,16 @@
         <v>602</v>
       </c>
       <c r="G26" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="H26" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I26" t="n">
-        <v>0.8183588981628418</v>
+        <v>1.423592805862427</v>
       </c>
       <c r="J26" t="n">
-        <v>0.8305647840531563</v>
+        <v>0.9966777408637874</v>
       </c>
     </row>
     <row r="27">
@@ -1508,16 +1508,16 @@
         <v>602</v>
       </c>
       <c r="G27" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="H27" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I27" t="n">
-        <v>0.8251771926879883</v>
+        <v>3.163264513015747</v>
       </c>
       <c r="J27" t="n">
-        <v>0.8305647840531563</v>
+        <v>0.9966777408637874</v>
       </c>
     </row>
     <row r="28">
@@ -1548,16 +1548,16 @@
         <v>482</v>
       </c>
       <c r="G28" t="n">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="H28" t="n">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="I28" t="n">
-        <v>0.8782398700714111</v>
+        <v>1.176267623901367</v>
       </c>
       <c r="J28" t="n">
-        <v>1.037344398340249</v>
+        <v>1.244813278008299</v>
       </c>
     </row>
     <row r="29">
@@ -1594,7 +1594,7 @@
         <v>488</v>
       </c>
       <c r="I29" t="n">
-        <v>0.7957446575164795</v>
+        <v>1.506341457366943</v>
       </c>
       <c r="J29" t="n">
         <v>1.0351966873706</v>
@@ -1628,16 +1628,16 @@
         <v>852</v>
       </c>
       <c r="G30" t="n">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="H30" t="n">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="I30" t="n">
-        <v>0.8416392803192139</v>
+        <v>1.29070782661438</v>
       </c>
       <c r="J30" t="n">
-        <v>0.5868544600938966</v>
+        <v>0.7042253521126761</v>
       </c>
     </row>
     <row r="31">
@@ -1668,16 +1668,16 @@
         <v>852</v>
       </c>
       <c r="G31" t="n">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="H31" t="n">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="I31" t="n">
-        <v>0.8689045906066895</v>
+        <v>1.28548526763916</v>
       </c>
       <c r="J31" t="n">
-        <v>0.5868544600938966</v>
+        <v>0.7042253521126761</v>
       </c>
     </row>
     <row r="32">
@@ -1714,7 +1714,7 @@
         <v>737</v>
       </c>
       <c r="I32" t="n">
-        <v>0.8861379623413086</v>
+        <v>2.624349594116211</v>
       </c>
       <c r="J32" t="n">
         <v>0.6830601092896175</v>
@@ -1748,16 +1748,16 @@
         <v>732</v>
       </c>
       <c r="G33" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="H33" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="I33" t="n">
-        <v>1.179498434066772</v>
+        <v>1.719299077987671</v>
       </c>
       <c r="J33" t="n">
-        <v>0.6830601092896175</v>
+        <v>0.819672131147541</v>
       </c>
     </row>
     <row r="34">
@@ -1788,16 +1788,16 @@
         <v>1228</v>
       </c>
       <c r="G34" t="n">
-        <v>1240</v>
+        <v>1247</v>
       </c>
       <c r="H34" t="n">
-        <v>1240</v>
+        <v>1247</v>
       </c>
       <c r="I34" t="n">
-        <v>3.606294393539429</v>
+        <v>3.559669017791748</v>
       </c>
       <c r="J34" t="n">
-        <v>0.9771986970684038</v>
+        <v>1.547231270358306</v>
       </c>
     </row>
     <row r="35">
@@ -1834,7 +1834,7 @@
         <v>1240</v>
       </c>
       <c r="I35" t="n">
-        <v>3.189956426620483</v>
+        <v>7.173325061798096</v>
       </c>
       <c r="J35" t="n">
         <v>0.8950366151342555</v>
@@ -1868,16 +1868,16 @@
         <v>984</v>
       </c>
       <c r="G36" t="n">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="H36" t="n">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="I36" t="n">
-        <v>3.300666332244873</v>
+        <v>15.6819474697113</v>
       </c>
       <c r="J36" t="n">
-        <v>1.016260162601626</v>
+        <v>1.117886178861789</v>
       </c>
     </row>
     <row r="37">
@@ -1914,7 +1914,7 @@
         <v>995</v>
       </c>
       <c r="I37" t="n">
-        <v>2.66900897026062</v>
+        <v>4.554160356521606</v>
       </c>
       <c r="J37" t="n">
         <v>1.117886178861789</v>
@@ -1948,16 +1948,16 @@
         <v>1728</v>
       </c>
       <c r="G38" t="n">
-        <v>1741</v>
+        <v>1747</v>
       </c>
       <c r="H38" t="n">
-        <v>1741</v>
+        <v>1747</v>
       </c>
       <c r="I38" t="n">
-        <v>2.885637998580933</v>
+        <v>19.68982005119324</v>
       </c>
       <c r="J38" t="n">
-        <v>0.7523148148148148</v>
+        <v>1.099537037037037</v>
       </c>
     </row>
     <row r="39">
@@ -1988,16 +1988,16 @@
         <v>1729</v>
       </c>
       <c r="G39" t="n">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="H39" t="n">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="I39" t="n">
-        <v>2.871102809906006</v>
+        <v>13.32058835029602</v>
       </c>
       <c r="J39" t="n">
-        <v>0.5205320994794679</v>
+        <v>0.6362058993637941</v>
       </c>
     </row>
     <row r="40">
@@ -2028,16 +2028,16 @@
         <v>1482</v>
       </c>
       <c r="G40" t="n">
-        <v>1496</v>
+        <v>1502</v>
       </c>
       <c r="H40" t="n">
-        <v>1496</v>
+        <v>1502</v>
       </c>
       <c r="I40" t="n">
-        <v>2.732436180114746</v>
+        <v>9.913250923156738</v>
       </c>
       <c r="J40" t="n">
-        <v>0.9446693657219973</v>
+        <v>1.349527665317139</v>
       </c>
     </row>
     <row r="41">
@@ -2074,7 +2074,7 @@
         <v>1495</v>
       </c>
       <c r="I41" t="n">
-        <v>2.928535461425781</v>
+        <v>17.61356973648071</v>
       </c>
       <c r="J41" t="n">
         <v>0.7412398921832885</v>
@@ -2108,16 +2108,16 @@
         <v>1820</v>
       </c>
       <c r="G42" t="n">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="H42" t="n">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="I42" t="n">
-        <v>5.903656244277954</v>
+        <v>53.68333292007446</v>
       </c>
       <c r="J42" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.3296703296703297</v>
       </c>
     </row>
     <row r="43">
@@ -2148,16 +2148,16 @@
         <v>1821</v>
       </c>
       <c r="G43" t="n">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="H43" t="n">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="I43" t="n">
-        <v>6.733601093292236</v>
+        <v>75.91025042533875</v>
       </c>
       <c r="J43" t="n">
-        <v>0.2196595277320154</v>
+        <v>0.2745744096650192</v>
       </c>
     </row>
     <row r="44">
@@ -2188,16 +2188,16 @@
         <v>1450</v>
       </c>
       <c r="G44" t="n">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="H44" t="n">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="I44" t="n">
-        <v>6.04203987121582</v>
+        <v>43.09460806846619</v>
       </c>
       <c r="J44" t="n">
-        <v>0.3448275862068966</v>
+        <v>0.4137931034482759</v>
       </c>
     </row>
     <row r="45">
@@ -2228,16 +2228,16 @@
         <v>1451</v>
       </c>
       <c r="G45" t="n">
-        <v>1456</v>
+        <v>1475</v>
       </c>
       <c r="H45" t="n">
-        <v>1456</v>
+        <v>1475</v>
       </c>
       <c r="I45" t="n">
-        <v>8.012970209121704</v>
+        <v>59.43610095977783</v>
       </c>
       <c r="J45" t="n">
-        <v>0.3445899379738112</v>
+        <v>1.654031702274293</v>
       </c>
     </row>
     <row r="46">
@@ -2268,16 +2268,16 @@
         <v>2571</v>
       </c>
       <c r="G46" t="n">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="H46" t="n">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="I46" t="n">
-        <v>7.240603923797607</v>
+        <v>79.67406058311462</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1944768572539868</v>
+        <v>0.2333722287047841</v>
       </c>
     </row>
     <row r="47">
@@ -2308,16 +2308,16 @@
         <v>2570</v>
       </c>
       <c r="G47" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="H47" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="I47" t="n">
-        <v>7.788285970687866</v>
+        <v>76.5239360332489</v>
       </c>
       <c r="J47" t="n">
-        <v>0.1945525291828794</v>
+        <v>0.2334630350194553</v>
       </c>
     </row>
     <row r="48">
@@ -2348,16 +2348,16 @@
         <v>2200</v>
       </c>
       <c r="G48" t="n">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="H48" t="n">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="I48" t="n">
-        <v>7.207762002944946</v>
+        <v>17.60400295257568</v>
       </c>
       <c r="J48" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.2727272727272728</v>
       </c>
     </row>
     <row r="49">
@@ -2388,16 +2388,16 @@
         <v>2200</v>
       </c>
       <c r="G49" t="n">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="H49" t="n">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="I49" t="n">
-        <v>5.751901388168335</v>
+        <v>52.23634195327759</v>
       </c>
       <c r="J49" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.2727272727272728</v>
       </c>
     </row>
     <row r="50">
@@ -2428,16 +2428,16 @@
         <v>2425</v>
       </c>
       <c r="G50" t="n">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="H50" t="n">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="I50" t="n">
-        <v>12.85013794898987</v>
+        <v>18.91699457168579</v>
       </c>
       <c r="J50" t="n">
-        <v>0.4948453608247422</v>
+        <v>0.6185567010309279</v>
       </c>
     </row>
     <row r="51">
@@ -2474,7 +2474,7 @@
         <v>2436</v>
       </c>
       <c r="I51" t="n">
-        <v>9.414394378662109</v>
+        <v>323.0808424949646</v>
       </c>
       <c r="J51" t="n">
         <v>0.3708281829419036</v>
@@ -2508,16 +2508,16 @@
         <v>1931</v>
       </c>
       <c r="G52" t="n">
-        <v>1938</v>
+        <v>1942</v>
       </c>
       <c r="H52" t="n">
-        <v>1938</v>
+        <v>1942</v>
       </c>
       <c r="I52" t="n">
-        <v>14.65603017807007</v>
+        <v>450.0036673545837</v>
       </c>
       <c r="J52" t="n">
-        <v>0.3625064733298809</v>
+        <v>0.5696530295183843</v>
       </c>
     </row>
     <row r="53">
@@ -2548,16 +2548,16 @@
         <v>1931</v>
       </c>
       <c r="G53" t="n">
-        <v>1959</v>
+        <v>1982</v>
       </c>
       <c r="H53" t="n">
-        <v>1959</v>
+        <v>1982</v>
       </c>
       <c r="I53" t="n">
-        <v>19.56046676635742</v>
+        <v>307.6818211078644</v>
       </c>
       <c r="J53" t="n">
-        <v>1.450025893319524</v>
+        <v>2.641118591403418</v>
       </c>
     </row>
     <row r="54">
@@ -2588,16 +2588,16 @@
         <v>3425</v>
       </c>
       <c r="G54" t="n">
-        <v>3436</v>
+        <v>3440</v>
       </c>
       <c r="H54" t="n">
-        <v>3436</v>
+        <v>3440</v>
       </c>
       <c r="I54" t="n">
-        <v>12.6053786277771</v>
+        <v>21908.05735230446</v>
       </c>
       <c r="J54" t="n">
-        <v>0.3211678832116788</v>
+        <v>0.4379562043795621</v>
       </c>
     </row>
     <row r="55">
@@ -2628,16 +2628,16 @@
         <v>3427</v>
       </c>
       <c r="G55" t="n">
-        <v>3433</v>
+        <v>3437</v>
       </c>
       <c r="H55" t="n">
-        <v>3433</v>
+        <v>3437</v>
       </c>
       <c r="I55" t="n">
-        <v>12.09920287132263</v>
+        <v>484.9503247737885</v>
       </c>
       <c r="J55" t="n">
-        <v>0.1750802451123432</v>
+        <v>0.2918004085205719</v>
       </c>
     </row>
     <row r="56">
@@ -2668,16 +2668,16 @@
         <v>2930</v>
       </c>
       <c r="G56" t="n">
-        <v>2940</v>
+        <v>2945</v>
       </c>
       <c r="H56" t="n">
-        <v>2940</v>
+        <v>2945</v>
       </c>
       <c r="I56" t="n">
-        <v>13.53523254394531</v>
+        <v>333.4353225231171</v>
       </c>
       <c r="J56" t="n">
-        <v>0.3412969283276451</v>
+        <v>0.5119453924914675</v>
       </c>
     </row>
     <row r="57">
@@ -2708,16 +2708,16 @@
         <v>2931</v>
       </c>
       <c r="G57" t="n">
-        <v>2937</v>
+        <v>2939</v>
       </c>
       <c r="H57" t="n">
-        <v>2937</v>
+        <v>2939</v>
       </c>
       <c r="I57" t="n">
-        <v>13.08927774429321</v>
+        <v>678.3832130432129</v>
       </c>
       <c r="J57" t="n">
-        <v>0.2047082906857728</v>
+        <v>0.2729443875810304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalizando plot gantt para VSN
</commit_message>
<xml_diff>
--- a/Resultados_atualizado.xlsx
+++ b/Resultados_atualizado.xlsx
@@ -507,18 +507,10 @@
       <c r="F2" t="n">
         <v>236</v>
       </c>
-      <c r="G2" t="n">
-        <v>236</v>
-      </c>
-      <c r="H2" t="n">
-        <v>236</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.1712169647216797</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -547,18 +539,10 @@
       <c r="F3" t="n">
         <v>238</v>
       </c>
-      <c r="G3" t="n">
-        <v>238</v>
-      </c>
-      <c r="H3" t="n">
-        <v>238</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.1421029567718506</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,18 +571,10 @@
       <c r="F4" t="n">
         <v>193</v>
       </c>
-      <c r="G4" t="n">
-        <v>193</v>
-      </c>
-      <c r="H4" t="n">
-        <v>193</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1716067790985107</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -634,7 +610,7 @@
         <v>193</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1861796379089355</v>
+        <v>164.1161313056946</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -667,18 +643,10 @@
       <c r="F6" t="n">
         <v>336</v>
       </c>
-      <c r="G6" t="n">
-        <v>336</v>
-      </c>
-      <c r="H6" t="n">
-        <v>336</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.1966288089752197</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,18 +675,10 @@
       <c r="F7" t="n">
         <v>338</v>
       </c>
-      <c r="G7" t="n">
-        <v>338</v>
-      </c>
-      <c r="H7" t="n">
-        <v>338</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.2164952754974365</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -747,18 +707,10 @@
       <c r="F8" t="n">
         <v>291</v>
       </c>
-      <c r="G8" t="n">
-        <v>291</v>
-      </c>
-      <c r="H8" t="n">
-        <v>291</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.144500732421875</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -787,18 +739,10 @@
       <c r="F9" t="n">
         <v>293</v>
       </c>
-      <c r="G9" t="n">
-        <v>293</v>
-      </c>
-      <c r="H9" t="n">
-        <v>293</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.1469166278839111</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -827,18 +771,10 @@
       <c r="F10" t="n">
         <v>355</v>
       </c>
-      <c r="G10" t="n">
-        <v>355</v>
-      </c>
-      <c r="H10" t="n">
-        <v>355</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.103016376495361</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -867,18 +803,10 @@
       <c r="F11" t="n">
         <v>355</v>
       </c>
-      <c r="G11" t="n">
-        <v>355</v>
-      </c>
-      <c r="H11" t="n">
-        <v>355</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.8459506034851074</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -907,18 +835,10 @@
       <c r="F12" t="n">
         <v>285</v>
       </c>
-      <c r="G12" t="n">
-        <v>285</v>
-      </c>
-      <c r="H12" t="n">
-        <v>285</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.7281584739685059</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -947,18 +867,10 @@
       <c r="F13" t="n">
         <v>285</v>
       </c>
-      <c r="G13" t="n">
-        <v>286</v>
-      </c>
-      <c r="H13" t="n">
-        <v>286</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.703357458114624</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.3508771929824561</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -987,18 +899,10 @@
       <c r="F14" t="n">
         <v>505</v>
       </c>
-      <c r="G14" t="n">
-        <v>505</v>
-      </c>
-      <c r="H14" t="n">
-        <v>505</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1.375955104827881</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1027,18 +931,10 @@
       <c r="F15" t="n">
         <v>505</v>
       </c>
-      <c r="G15" t="n">
-        <v>506</v>
-      </c>
-      <c r="H15" t="n">
-        <v>506</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.8674395084381104</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.198019801980198</v>
-      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1067,18 +963,10 @@
       <c r="F16" t="n">
         <v>435</v>
       </c>
-      <c r="G16" t="n">
-        <v>435</v>
-      </c>
-      <c r="H16" t="n">
-        <v>435</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.392467975616455</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1107,18 +995,10 @@
       <c r="F17" t="n">
         <v>435</v>
       </c>
-      <c r="G17" t="n">
-        <v>435</v>
-      </c>
-      <c r="H17" t="n">
-        <v>435</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.9371294975280762</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1147,18 +1027,10 @@
       <c r="F18" t="n">
         <v>481</v>
       </c>
-      <c r="G18" t="n">
-        <v>482</v>
-      </c>
-      <c r="H18" t="n">
-        <v>482</v>
-      </c>
-      <c r="I18" t="n">
-        <v>2.936053276062012</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.2079002079002079</v>
-      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1187,18 +1059,10 @@
       <c r="F19" t="n">
         <v>481</v>
       </c>
-      <c r="G19" t="n">
-        <v>482</v>
-      </c>
-      <c r="H19" t="n">
-        <v>482</v>
-      </c>
-      <c r="I19" t="n">
-        <v>6.35129451751709</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.2079002079002079</v>
-      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1227,18 +1091,10 @@
       <c r="F20" t="n">
         <v>386</v>
       </c>
-      <c r="G20" t="n">
-        <v>388</v>
-      </c>
-      <c r="H20" t="n">
-        <v>388</v>
-      </c>
-      <c r="I20" t="n">
-        <v>3.332239866256714</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.5181347150259068</v>
-      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1267,18 +1123,10 @@
       <c r="F21" t="n">
         <v>386</v>
       </c>
-      <c r="G21" t="n">
-        <v>389</v>
-      </c>
-      <c r="H21" t="n">
-        <v>389</v>
-      </c>
-      <c r="I21" t="n">
-        <v>3.640355110168457</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.7772020725388601</v>
-      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1307,18 +1155,10 @@
       <c r="F22" t="n">
         <v>681</v>
       </c>
-      <c r="G22" t="n">
-        <v>683</v>
-      </c>
-      <c r="H22" t="n">
-        <v>683</v>
-      </c>
-      <c r="I22" t="n">
-        <v>2.783428192138672</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.2936857562408223</v>
-      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1347,18 +1187,10 @@
       <c r="F23" t="n">
         <v>681</v>
       </c>
-      <c r="G23" t="n">
-        <v>682</v>
-      </c>
-      <c r="H23" t="n">
-        <v>682</v>
-      </c>
-      <c r="I23" t="n">
-        <v>4.972759008407593</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.1468428781204112</v>
-      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1387,18 +1219,10 @@
       <c r="F24" t="n">
         <v>586</v>
       </c>
-      <c r="G24" t="n">
-        <v>587</v>
-      </c>
-      <c r="H24" t="n">
-        <v>587</v>
-      </c>
-      <c r="I24" t="n">
-        <v>2.694021701812744</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.1706484641638225</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1427,18 +1251,10 @@
       <c r="F25" t="n">
         <v>586</v>
       </c>
-      <c r="G25" t="n">
-        <v>587</v>
-      </c>
-      <c r="H25" t="n">
-        <v>587</v>
-      </c>
-      <c r="I25" t="n">
-        <v>4.272587060928345</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.1706484641638225</v>
-      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1467,18 +1283,10 @@
       <c r="F26" t="n">
         <v>602</v>
       </c>
-      <c r="G26" t="n">
-        <v>605</v>
-      </c>
-      <c r="H26" t="n">
-        <v>605</v>
-      </c>
-      <c r="I26" t="n">
-        <v>8.249611139297485</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.4983388704318937</v>
-      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1507,18 +1315,10 @@
       <c r="F27" t="n">
         <v>602</v>
       </c>
-      <c r="G27" t="n">
-        <v>604</v>
-      </c>
-      <c r="H27" t="n">
-        <v>604</v>
-      </c>
-      <c r="I27" t="n">
-        <v>11.18136191368103</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.3322259136212625</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1547,18 +1347,10 @@
       <c r="F28" t="n">
         <v>482</v>
       </c>
-      <c r="G28" t="n">
-        <v>483</v>
-      </c>
-      <c r="H28" t="n">
-        <v>483</v>
-      </c>
-      <c r="I28" t="n">
-        <v>16.07267379760742</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.2074688796680498</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1587,18 +1379,10 @@
       <c r="F29" t="n">
         <v>483</v>
       </c>
-      <c r="G29" t="n">
-        <v>484</v>
-      </c>
-      <c r="H29" t="n">
-        <v>484</v>
-      </c>
-      <c r="I29" t="n">
-        <v>10.19558453559875</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.2070393374741201</v>
-      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1627,18 +1411,10 @@
       <c r="F30" t="n">
         <v>852</v>
       </c>
-      <c r="G30" t="n">
-        <v>854</v>
-      </c>
-      <c r="H30" t="n">
-        <v>854</v>
-      </c>
-      <c r="I30" t="n">
-        <v>11.59835171699524</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.2347417840375587</v>
-      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1667,18 +1443,10 @@
       <c r="F31" t="n">
         <v>852</v>
       </c>
-      <c r="G31" t="n">
-        <v>855</v>
-      </c>
-      <c r="H31" t="n">
-        <v>855</v>
-      </c>
-      <c r="I31" t="n">
-        <v>8.783922910690308</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.3521126760563381</v>
-      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1707,18 +1475,10 @@
       <c r="F32" t="n">
         <v>732</v>
       </c>
-      <c r="G32" t="n">
-        <v>733</v>
-      </c>
-      <c r="H32" t="n">
-        <v>733</v>
-      </c>
-      <c r="I32" t="n">
-        <v>14.91614294052124</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0.1366120218579235</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1747,18 +1507,10 @@
       <c r="F33" t="n">
         <v>732</v>
       </c>
-      <c r="G33" t="n">
-        <v>734</v>
-      </c>
-      <c r="H33" t="n">
-        <v>734</v>
-      </c>
-      <c r="I33" t="n">
-        <v>15.8888955116272</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0.273224043715847</v>
-      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">

</xml_diff>